<commit_message>
Add automatic quality validation for pipeline outputs
- Add QualityReport dataclass with success rate, quality score, and issue detection
- Add validate_output_quality() method to ExecutionResult
- CLI now automatically validates output quality after processing
- SDK/scripts can call result.validate_output_quality() for validation
- Quality thresholds: excellent (95%+), good (80%+), poor (50%+), critical (<50%)
- Raises warnings when success rate < 70% (unacceptable quality)
- Detects metrics mismatch (pipeline reports 0 failures but nulls exist)
- Provides actionable recommendations for quality issues
- Simplified bacon_cleaning_config.yaml prompt (matches SDK for consistency)
</commit_message>
<xml_diff>
--- a/tmp/bacon_all_365_cleaned.xlsx
+++ b/tmp/bacon_all_365_cleaned.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Applewood-smoked half-slab and slab bacon.</t>
+          <t>Applewood-smoked half-slab and slab bacon</t>
         </is>
       </c>
     </row>
@@ -592,11 +592,7 @@
           <t>FRZ PRE-CKD BCN SAND STYLE 300 | BACON SAND STYLE CKD</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Frozen pre-cooked sandwich-style bacon</t>
-        </is>
-      </c>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -624,7 +620,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cooked gas‑flushed bacon pieces, .375‑inch; fully cooked gluten‑free bacon bits, 3/8‑inch.</t>
+          <t>Cooked gas‑flushed bacon pieces, .375‑inch, and fully cooked gluten‑free bacon bits, 3/8‑inch.</t>
         </is>
       </c>
     </row>
@@ -639,11 +635,7 @@
           <t>BACON BITS REAL GAS FLUSHED .75 IN | BACON BIT REAL COOKED GLUTEN FREE 3/4"" | BACON BIT REAL CKD 3/4IN GF</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Fully cooked gluten-free bacon bits, 3/4‑inch pieces</t>
-        </is>
-      </c>
+      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -658,7 +650,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 3/8-inch pieces</t>
+          <t>Fully cooked diced bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -675,7 +667,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Sliced smoked bacon, 18-22 slices per pound, layflat</t>
+          <t>Smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -692,7 +684,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fully cooked finely diced bacon bits.</t>
+          <t>Fully cooked finely diced bacon bits</t>
         </is>
       </c>
     </row>
@@ -790,7 +782,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Applewood cold-smoked sliced bacon, 10-12 slices per pound, gluten-free.</t>
+          <t>Gluten-free applewood cold-smoked sliced bacon, 10-12 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -822,11 +814,7 @@
           <t>BACN,BITS,FC,SMFD,1/4IN,2/5# | BACON BIT 1/4IN FC | BACON BIT FULLY COOKED 1/4""</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Fully cooked bacon bits, 1/4-inch pieces.</t>
-        </is>
-      </c>
+      <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -852,7 +840,11 @@
           <t>BCN,ARM,2/5#,3/4",FLCK,TPG | BACON TOPPING REAL FC 3/4""</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Fully cooked flaked bacon topping, 3/4‑inch pieces</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -895,11 +887,7 @@
           <t>GFS SLCD BACN 9/11 | BACON SLCD 9-11CT FRSH</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Raw sliced bacon, 9-11 slices per pound</t>
-        </is>
-      </c>
+      <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -914,7 +902,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Cooked sliced bacon, 18-22 slices per pound</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -944,7 +932,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Cooked thick-cut sliced applewood-smoked bacon.</t>
+          <t>Cooked thick-cut sliced applewood-smoked bacon</t>
         </is>
       </c>
     </row>
@@ -961,7 +949,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 1/2‑inch pieces</t>
+          <t>Fully cooked bacon bits, 1/2-inch pieces</t>
         </is>
       </c>
     </row>
@@ -989,11 +977,7 @@
           <t>JMYD FC AWS SLCD BACN 4/150 | BACON PRECOOKED APPLWOOD 10 IN</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Fully cooked applewood-smoked sliced bacon, 10‑inch slices</t>
-        </is>
-      </c>
+      <c r="C35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1025,7 +1009,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Fully cooked half-sliced bacon</t>
+          <t>Fully cooked half-sliced bacon, 576 slices</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1026,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Fully cooked half-sliced bacon, 18-22 slices per pound</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1056,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Raw diced bacon bits</t>
+          <t>Raw diced bacon pieces</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1107,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Frozen sliced hickory-smoked bacon, 18-22 slices per pound, layflat</t>
+          <t>Frozen hickory-smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1219,11 +1203,7 @@
           <t>NT HKY SMKD THK SLCD BULK BACN 5/INCH FZ | BACON BULK SLI THCK HCKRY SMK</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Frozen sliced thick hickory-smoked bacon</t>
-        </is>
-      </c>
+      <c r="C49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1249,7 +1229,11 @@
           <t>NT AWS BACN FPK 14/18, GF | BACON LAYFLAT 14/18 APPL GF</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Gluten-free applewood-smoked</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1311,7 +1295,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 192 slices per package</t>
+          <t>Fully cooked sliced bacon, 192 pieces</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1312,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Raw cured sliced smoked bacon, 18-22 slices per pound, layflat</t>
+          <t>Raw sliced smoked bacon, 18-22</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1346,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Gluten-free sliced slab bacon, 9-13 slices per pound.</t>
+          <t>Sliced slab bacon, 9-13 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1427,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Sliced layflat bacon, 18-22 slices per pound.</t>
+          <t>Layflat sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1444,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Sliced bacon, 16-18 slices per pound</t>
+          <t>Shingle bacon, 16-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1461,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Frozen sliced applewood-smoked bacon, 10-12 slices per pound.</t>
+          <t>Frozen applewood-smoked sliced bacon, 10-12 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1495,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Fully cooked bacon pieces, 1/2‑inch pieces</t>
+          <t>Fully cooked bacon pieces, 1/2-inch pieces</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1529,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Applewood-smoked cubed and diced bacon, 0.5 × 0.5‑inch pieces.</t>
+          <t>Applewood-smoked cubed bacon, 0.5 × 0.5‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1557,11 @@
           <t>BACON PIECES COOKED GAS FLUSHED .375 IN | BACON BIT REAL CKD 3/8 GF | BACON BIT REAL COOKED GLUTEN FREE 3/8""</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Cooked gas‑flushed bacon pieces, .375‑inch, and fully cooked gluten‑free bacon bits, 3/8‑inch.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1588,7 +1576,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 0.5‑inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 1/2-inch pieces</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1640,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Raw sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1657,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Raw sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1704,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Fully cooked thin sliced bacon</t>
+          <t>Fully cooked thin sliced bacon.</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1862,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Fully cooked diced bacon topping, 3/8‑inch pieces</t>
+          <t>Fully cooked diced bacon topping, 3/8‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1896,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits,</t>
+          <t>Fully cooked diced bacon bits, 0.375‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1913,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 300 slices per case</t>
+          <t>Fully cooked sliced bacon, 300 slices per case.</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1947,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 300 slices per case</t>
+          <t>Fully cooked sliced bacon, 300 slices per case.</t>
         </is>
       </c>
     </row>
@@ -2008,7 +1996,11 @@
           <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND | BACON LAYFLAT C/C 18/22 SMK GF</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Gluten-free smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2125,7 +2117,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Gluten-free applewood-smoked sliced bacon, 13-17 slices per pound, layflat.</t>
         </is>
       </c>
     </row>
@@ -2159,7 +2151,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Half-stick Canadian-style bacon</t>
+          <t>Canadian-style half-stick bacon.</t>
         </is>
       </c>
     </row>
@@ -2176,7 +2168,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Canadian-style whole bacon sticks</t>
+          <t>Canadian-style whole stick bacon</t>
         </is>
       </c>
     </row>
@@ -2259,11 +2251,7 @@
           <t>BACON CUBED COOKED .25X.25 | BACON TOPPING CKD 1/4IN DCD | BACON COOKED DICED 1/4""</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>Cooked bacon topping, 1/4‑inch diced cubes.</t>
-        </is>
-      </c>
+      <c r="C113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2278,7 +2266,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Thick-cut sliced bacon, 1/2-inch slices</t>
+          <t>Thick-cut sliced bacon, 1/2-inch slices.</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2283,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon and fully cooked slab bacon</t>
+          <t>Fully cooked sliced and slab bacon</t>
         </is>
       </c>
     </row>
@@ -2434,11 +2422,7 @@
           <t>BACON L/O #2 FZ 15# P/L | BACON L/O #2 FZ CHEF'S CHC | BACON #2 LAYOUT FROZEN</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>Frozen sliced bacon, layflat</t>
-        </is>
-      </c>
+      <c r="C124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2451,11 +2435,7 @@
           <t>BACON SLICED APPLEWOOD LAYFLAT GAS FLUSHED PRIME12 14-16 CT | BACON LAYFLT 14/16 AW GF PR12</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Applewood-smoked sliced bacon, gluten-free, 14-16 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -2487,7 +2467,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Fully cooked thin sliced bacon and fully cooked medium sliced bacon</t>
+          <t>Fully cooked thin and medium sliced bacon</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2484,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Fully cooked medium-sliced and thin-sliced bacon.</t>
+          <t>Fully cooked medium-sliced bacon and fully cooked thin-sliced bacon.</t>
         </is>
       </c>
     </row>
@@ -2619,11 +2599,7 @@
           <t>BACON BEEF SLICED SMOKED HONEY CURED RAW | BACON BEEF SLAB SLICE</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>Raw honey-cured smoked sliced bacon, slab bacon</t>
-        </is>
-      </c>
+      <c r="C135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2685,7 +2661,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Sliced extra‑thick bacon, 14‑18 slices per pound</t>
+          <t>Extra-thick sliced bacon, 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2678,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Maple pepper sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Sliced bacon, 13-17 slices per pound, layflat.</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2695,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Raw gluten-free smoked sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Gluten-free smoked sliced bacon, 13-17 slices per</t>
         </is>
       </c>
     </row>
@@ -2736,7 +2712,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Water-added Canadian-style bacon with sirloin.</t>
+          <t>Water-added Canadian-style bacon with sirloin</t>
         </is>
       </c>
     </row>
@@ -2768,7 +2744,11 @@
           <t>HORMEL HONEY CURED BACON 13 17 SLICES PER POUND WIDE SHINGLE | BACON LAYFLAT E/E 13/17 HNY GF</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr"/>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Honey-cured sliced bacon, 13-17 slices per pound, gluten-free, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2800,7 +2780,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Honey-cured gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Honey-cured sliced bacon, 18-22 slices per pound, gluten-free, layflat</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2797,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon topping, 1/2‑inch slices</t>
+          <t>Fully cooked sliced topping bacon, 1/2-inch slices.</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Cooked bacon topping, 1/2-inch pieces</t>
+          <t>Fully cooked bacon topping, 0.5-inch pieces</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2848,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 9‑13 slices per pound, layflat.</t>
+          <t>Applewood-smoked sliced bacon, 9-13 slices per pound, gluten-free, layflat</t>
         </is>
       </c>
     </row>
@@ -2919,7 +2899,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Fully cooked uncured sliced bacon, 13-17 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -2936,7 +2916,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Raw uncured sliced bacon, 13-17 slices per pound, gluten‑free, layflat</t>
+          <t>Uncured natural gluten-free sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2933,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Canadian-style sliced and quartered bacon, 10 slices per ounce</t>
+          <t>Sliced and quartered Canadian-style bacon, 10 slices per ounce.</t>
         </is>
       </c>
     </row>
@@ -2970,7 +2950,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Fully cooked bacon pieces, 1/2-inch pieces</t>
+          <t>Fully cooked bacon pieces, 1/2‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -3004,7 +2984,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Fully cooked sugar-cured thick sliced bacon</t>
+          <t>Fully cooked thick sliced sugar-cured bacon</t>
         </is>
       </c>
     </row>
@@ -3019,11 +2999,7 @@
           <t>HORMEL BLACK LABEL BACON 13 17 PIECES PER POUND | BACON SLAB CC 13/17 SMK BLK GF</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>Gluten-free black-smoked slab bacon, 13-17 slices per pound.</t>
-        </is>
-      </c>
+      <c r="C159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3055,7 +3031,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Frozen sliced jalapeño bacon, 13-17 slices per pound, layflat</t>
+          <t>Frozen jalapeno-flavored sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3170,7 +3146,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Bacon cheeseburger with bacon on brioche bun</t>
+          <t>Bacon cheeseburger on brioche bun</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3163,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Sliced bacon</t>
+          <t>Raw sliced beef bacon</t>
         </is>
       </c>
     </row>
@@ -3202,11 +3178,7 @@
           <t>HORMEL LAYOUT BACON 23 27 SLICES PER POUND | BACON LAYFLAT C/C 23/27 SMK GF</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>Gluten-free smoked sliced bacon, 23-27 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -3221,7 +3193,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon topping, 1‑inch pieces</t>
+          <t>Fully cooked bacon topping, 1‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3240,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Fully cooked applewood-smoked diced bacon.</t>
+          <t>Fully cooked diced applewood-smoked bacon pieces</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3289,11 @@
           <t>8 SYS HKSM LFLT SLCD BACN 18/22 GF 15 LB | BACON LAYFLT 18/22 SMK GF PR12</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr"/>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Gluten-free hickory-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -3400,7 +3376,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Fully cooked smoked sliced bacon.</t>
+          <t>Fully cooked smoked sliced bacon</t>
         </is>
       </c>
     </row>
@@ -3447,7 +3423,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Center cut Texas-smoked sliced slab bacon, 18-22 slices per pound</t>
+          <t>Texas-smoked sliced slab bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -3464,7 +3440,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Smoked sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Smoked sliced layflat bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -3479,11 +3455,7 @@
           <t>SYS 1359413 LYFLT BACNSYSCO CLASSIC TEXAS SMKD CTCT INDIVIDUAL SPACED, LAYFLAT BACON (14/18) 1/15# | BACON LAYFLAT CC 14/18 TX SMKD</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>Texas-smoked layflat sliced bacon, 14-18 slices per pound.</t>
-        </is>
-      </c>
+      <c r="C187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -3515,7 +3487,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Texas-smoked sliced slab bacon, 14-18 slices per pound</t>
+          <t>Texas-smoked sliced bacon, 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3504,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 3/4-inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 3/4‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -3562,7 +3534,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 24-26 slices per pound, and thick-slice bacon</t>
+          <t>Fully cooked sliced bacon, 24-26 slices per pound; thick-slice bacon</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3551,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 3/8‑inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 3/8-inch pieces</t>
         </is>
       </c>
     </row>
@@ -3596,7 +3568,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Hardwood-smoked sliced rolled pork belly bacon.</t>
+          <t>Hardwood-smoked sliced rolled pork belly.</t>
         </is>
       </c>
     </row>
@@ -3613,7 +3585,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Texas-smoked sliced layflat bacon, 18-22 slices per pound</t>
+          <t>Texas-smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3630,7 +3602,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Fruitwood- and applewood-smoked slab bacon</t>
+          <t>Fruitwood-smoked slab bacon, 12 per pound; applewood-smoked slab bacon, 12 per pound</t>
         </is>
       </c>
     </row>
@@ -3645,11 +3617,7 @@
           <t>SYS 1345669 SLAB BACNCLASSIC TEXAS SMOKED CENTER CUT SLICED SLAB BACON (10/14) 1/15# | BACON SLAB C/C 10/14 TX SMOKED</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>Raw center-cut sliced slab bacon, Texas-smoked</t>
-        </is>
-      </c>
+      <c r="C197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -3692,11 +3660,7 @@
           <t>FRZ 1151422 REL LF 14/18 15LB | BACON 14/18 CT LAYFLAT E/E SMOKED</t>
         </is>
       </c>
-      <c r="C200" t="inlineStr">
-        <is>
-          <t>Frozen sliced bacon, 14-18 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -3711,7 +3675,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Frozen smoked sliced bacon, 22-26 slices per pound, layflat</t>
+          <t>Frozen sliced smoked bacon, 22-26 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3728,7 +3692,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Sliced pork bacon, 18-22 slices per pound, layflat</t>
+          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3709,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Bacon</t>
+          <t>Bacon.</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3794,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Bacon egg and cheese bowl</t>
+          <t>Bacon, egg, and cheese bowl</t>
         </is>
       </c>
     </row>
@@ -3864,7 +3828,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 300 slices per pound</t>
+          <t>Fully cooked sliced bacon, 300 slices</t>
         </is>
       </c>
     </row>
@@ -3932,7 +3896,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Hardwood-smoked bacon with apple cider flavor, gluten‑free.</t>
+          <t>Gluten-free hardwood-smoked bacon with apple cider.</t>
         </is>
       </c>
     </row>
@@ -3949,7 +3913,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Frozen applewood-smoked slab bacon, 10-12 slices per pound.</t>
+          <t>Frozen applewood-smoked slab bacon, 10-12 pieces per pound.</t>
         </is>
       </c>
     </row>
@@ -4000,7 +3964,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Bacon puree</t>
+          <t>Bacon puree.</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4015,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Smoked sliced bacon, layflat.</t>
+          <t>Smoked sliced layflat bacon.</t>
         </is>
       </c>
     </row>
@@ -4068,7 +4032,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Raw sliced wide shingled applewood-smoked bacon, 13-17 slices per pound</t>
+          <t>Raw wide shingled sliced applewood-smoked bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4049,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Raw wide shingled sliced applewood-smoked bacon, 13-17 slices per pound, layflat.</t>
+          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4102,7 +4066,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Raw wide shingled sliced applewood-smoked bacon, 13-17 slices per pound, layflat</t>
+          <t>Raw sliced applewood-smoked bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4119,7 +4083,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Applewood-smoked sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4136,7 +4100,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Raw sliced applewood-smoked bacon, 18-22 slices per pound, layflat</t>
+          <t>Raw gluten-free sliced applewood-smoked bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4132,11 @@
           <t>FRZ SUG TWO STAR EZ 14/18 | BACON LAY FLAT SMKD 14-18CT</t>
         </is>
       </c>
-      <c r="C228" t="inlineStr"/>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Frozen sugar-cured smoked sliced bacon, 14-18 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -4181,7 +4149,11 @@
           <t>HORMEL NATURAL CHOICE UNCURED BACON 18 22 SLICES PER POUND | BACON LAYFLAT C/C 18/22 NTGF F</t>
         </is>
       </c>
-      <c r="C229" t="inlineStr"/>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Raw uncured sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -4196,7 +4168,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Raw uncured sliced bacon, 18-22 slices per pound, gluten-free, layflat</t>
+          <t>Raw uncured natural gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4258,11 +4230,7 @@
           <t>BACON SLAB SLI 16/18 CT FRZN | BACON 16/18 CT SLAB HARDWOOD SMOKED SLICED</t>
         </is>
       </c>
-      <c r="C234" t="inlineStr">
-        <is>
-          <t>Frozen sliced slab bacon, hardwood-smoked, 16-18 slices per pound</t>
-        </is>
-      </c>
+      <c r="C234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -4294,7 +4262,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 16-18 slices per pound, layflat</t>
+          <t>Applewood-smoked bacon, 16-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4373,7 +4341,11 @@
           <t>SYS 5886381 APLEWD BACNSYSCO CLS GRILL FRESH APPLEWOOD SMOKED SLICED BACON 14/18 2/10# | BACON LAYFLAT C/C 14/18 APL GF</t>
         </is>
       </c>
-      <c r="C241" t="inlineStr"/>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Raw gluten-free applewood-smoked sliced bacon, 14-18 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -4388,7 +4360,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Fully cooked thick sliced bacon</t>
+          <t>Fully cooked thick sliced and slab bacon</t>
         </is>
       </c>
     </row>
@@ -4403,11 +4375,7 @@
           <t>BACON SLICED HONEY CURED 18-20 CT | BACON SHINGLE C/C 18/20 HNY</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>Honey-cured sliced bacon, 18-20 slices per pound</t>
-        </is>
-      </c>
+      <c r="C243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -4437,11 +4405,7 @@
           <t>BACON SLICED HONEY CURED 10-12 CT | BACON SHINGLE C/C 10/12 HNY</t>
         </is>
       </c>
-      <c r="C245" t="inlineStr">
-        <is>
-          <t>Honey-cured sliced bacon, 10-12 slices per pound.</t>
-        </is>
-      </c>
+      <c r="C245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -4480,11 +4444,7 @@
           <t>BACON SLICED APPLEWOOD SMOKED 14-18 CT | BACON LAYFLAT C/C 14/18 APL GF</t>
         </is>
       </c>
-      <c r="C248" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 14-18 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -4514,11 +4474,7 @@
           <t>BACON SLICED SUGAR CURED 14-16 CT | BACON SHINGLE C/C 14/16 SGR</t>
         </is>
       </c>
-      <c r="C250" t="inlineStr">
-        <is>
-          <t>Sugar-cured sliced and shingle bacon, 14-16 slices per pound</t>
-        </is>
-      </c>
+      <c r="C250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -4574,11 +4530,7 @@
           <t>BACON SLICED COOKED 10-12 CT | BACON PRECOOKED SLI THICK 2XX</t>
         </is>
       </c>
-      <c r="C254" t="inlineStr">
-        <is>
-          <t>Fully cooked thick sliced bacon, 10-12 slices per pound</t>
-        </is>
-      </c>
+      <c r="C254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -4606,7 +4558,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Natural hickory-smoked sliced bacon, 14-18 slices per pound.</t>
+          <t>Hickory-smoked sliced bacon, 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4683,7 +4635,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Cubed bacon chips, 0.375 × 0.375‑inch pieces</t>
+          <t>Raw cubed bacon chips, 0.375 × 0.375 in pieces, and diced real pork bacon, 0.38 in pieces.</t>
         </is>
       </c>
     </row>
@@ -4700,7 +4652,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Fully cooked diced bacon chips, 3/8-inch pieces</t>
+          <t>Fully cooked diced bacon chips, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -4732,11 +4684,7 @@
           <t>FRZ 5757184 REL SLAB 14/18 15# | BACON SLAB 14/18 SMOKED | BACON 14/18 CT SLAB SLICED</t>
         </is>
       </c>
-      <c r="C264" t="inlineStr">
-        <is>
-          <t>Frozen smoked slab bacon, 14-18 slices per pound.</t>
-        </is>
-      </c>
+      <c r="C264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -4749,11 +4697,7 @@
           <t>5886579 CLASSIC GRL/FRSH 14/18 | BACON LAYFLAT C/C 14/18 SMK GF</t>
         </is>
       </c>
-      <c r="C265" t="inlineStr">
-        <is>
-          <t>Fresh gluten-free sliced bacon, 14-18 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -4815,7 +4759,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 9-13 slices per pound.</t>
+          <t>Applewood-smoked sliced bacon, 9-13 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4789,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Cooked cubed bacon, 0.75 × 0.75‑inch pieces, and diced bacon, 3/4‑inch pieces.</t>
+          <t>Cooked cubed bacon, 0.75 × 0.75‑inch pieces; diced bacon, 3/4‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -4862,7 +4806,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Frozen applewood-smoked sliced slab bacon, 14-18 slices per pound</t>
+          <t>Frozen applewood-smoked slab bacon, 14-18 slices</t>
         </is>
       </c>
     </row>
@@ -4896,7 +4840,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Applewood-smoked slab sliced bacon, 1/4‑inch slices</t>
+          <t>Applewood-smoked slab sliced bacon, 1/4‑inch slices.</t>
         </is>
       </c>
     </row>
@@ -4947,7 +4891,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Fully cooked diced bacon, 1/2‑inch pieces, topping.</t>
+          <t>Fully cooked diced bacon, 1/2‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -4962,7 +4906,11 @@
           <t>10 LB CWA BULK BACN10 LBS SLICED BACON (PORK) BULK | BACON SLAB RANDOM SMOKED #2</t>
         </is>
       </c>
-      <c r="C278" t="inlineStr"/>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Raw sliced and slab bacon, random-smoked</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -4975,11 +4923,7 @@
           <t>WRGHT FPK BACN 15 LB FZNATURAL HICKORY SMOKED REGULAR FLAT PACK BACON. 15# FROZEN | BACON LAYFLAT 14/18 CT</t>
         </is>
       </c>
-      <c r="C279" t="inlineStr">
-        <is>
-          <t>Frozen sliced hickory-smoked bacon, 14-18 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -4994,7 +4938,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Fully cooked smoked sliced bacon, 20-24 slices per pound</t>
+          <t>Fully cooked smoked sliced bacon, 20-24 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5045,7 +4989,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked slab bacon, 14-16 slices per pound</t>
+          <t>Gluten-free applewood-smoked slab bacon, 14-16 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5073,11 +5017,7 @@
           <t>SYS 0855195 HON 10/12SYSCO CLASSIC BACON CENTER CUT SHINGLE HONEY 10/12 CT 1/15 LB | BACON SHINGLE C/C 10/12 HNY GF</t>
         </is>
       </c>
-      <c r="C285" t="inlineStr">
-        <is>
-          <t>Raw honey-glazed center cut shingle bacon, gluten-free, 10-12 slices per pound</t>
-        </is>
-      </c>
+      <c r="C285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -5092,7 +5032,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 16-18 slices per pound</t>
+          <t>Applewood-smoked sliced bacon, 16-18 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5143,7 +5083,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Fully cooked smoked bacon, 13-17 slices per pound.</t>
+          <t>Fully cooked smoked sliced bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5177,7 +5117,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5194,7 +5134,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5211,7 +5151,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Fresh gluten-free sliced bacon, 18-22 slices per pound.</t>
+          <t>Fresh gluten-free sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5311,7 +5251,11 @@
           <t>BCN,FL,BM,2/1.25#,300C,FLCK,SLCD | BACON LAYFLAT PRCK</t>
         </is>
       </c>
-      <c r="C299" t="inlineStr"/>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Fully cooked sliced bacon, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -5324,7 +5268,11 @@
           <t>BCN,FL,BM,2/1.25#,300C,FLCK,SLCD | BACON FULLY CKD HEAT N SERVE</t>
         </is>
       </c>
-      <c r="C300" t="inlineStr"/>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Fully cooked sliced bacon</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -5356,7 +5304,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices</t>
+          <t>Sliced bacon, 18-</t>
         </is>
       </c>
     </row>
@@ -5373,7 +5321,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound</t>
+          <t>Sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5448,11 +5396,7 @@
           <t>BCN,JM,APLWD,14/17/SLC,GF,1/15# | BACON 14/17 CT APPLEWOOD SMOKED SINGLE SHINGLE</t>
         </is>
       </c>
-      <c r="C308" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 14-17 slices per pound</t>
-        </is>
-      </c>
+      <c r="C308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -5510,7 +5454,7 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 3/16-inch pieces</t>
+          <t>Fully cooked fine bacon bits, 3/16‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -5527,7 +5471,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Ready-to-cook diced bacon; raw diced bacon ends and pieces, 1/2‑inch pieces</t>
+          <t>Ready-to-cook diced bacon and raw diced bacon ends</t>
         </is>
       </c>
     </row>
@@ -5578,7 +5522,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Fully cooked applewood-smoked bacon topping bits, 3/8-inch pieces</t>
+          <t>Fully cooked applewood-smoked bacon topping, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -5610,7 +5554,11 @@
           <t>BACN,SS,LS,GM,18/22,GF,15#,Z | BACON LAYFLAT C/C 18/22 LS</t>
         </is>
       </c>
-      <c r="C318" t="inlineStr"/>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -5649,7 +5597,11 @@
           <t>BCN,FL,RMP,1/15#,SS,GRDOUT,FZ | BACON 18/22 CT SINGLE SLICE IRREGULAR #2</t>
         </is>
       </c>
-      <c r="C321" t="inlineStr"/>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Frozen sliced bacon, 18-22 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -5662,7 +5614,11 @@
           <t>BACN,SS,SM,14/18,15#,Z | BACON SINGLE SLI 14/18 FRZN | BACON 14/18 CT SINGLE SLICE 70247158247</t>
         </is>
       </c>
-      <c r="C322" t="inlineStr"/>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Frozen single-slice bacon, 14-18 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -5675,11 +5631,7 @@
           <t>BACN,SS,SM,14/18,15#,Z | BACON 14/18 CT SINGLE SLICE 70247158247</t>
         </is>
       </c>
-      <c r="C323" t="inlineStr">
-        <is>
-          <t>Smoked sliced bacon, 14-18</t>
-        </is>
-      </c>
+      <c r="C323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -5694,7 +5646,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Raw smoked sliced bacon, 14-18 slices per</t>
+          <t>Raw sliced bacon, 14-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -5711,7 +5663,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, 18-22 slices</t>
+          <t>Frozen sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -5726,11 +5678,7 @@
           <t>BCN,FL,SMD,1/15#,18-22SL/#,FZ | BACON 18/22 CT LAYOUT SINGLE SLICED GLUTEN-FREE | BACON LAYOUT 18/22 SLVR MEDAL</t>
         </is>
       </c>
-      <c r="C326" t="inlineStr">
-        <is>
-          <t>Frozen gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -5786,11 +5734,7 @@
           <t>BACN,SS,SM,18/22,GF,15# | BACON SSL 18-22 | BACON 18/22 CT SINGLE SLICE GAS FLUSHED</t>
         </is>
       </c>
-      <c r="C330" t="inlineStr">
-        <is>
-          <t>Gluten</t>
-        </is>
-      </c>
+      <c r="C330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -5805,7 +5749,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Gluten-free Northwest-smoked sliced bacon, 10-14 slices per pound.</t>
+          <t>Gluten-free sliced bacon, Northwest-smoked, 10-14 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5872,11 +5816,7 @@
           <t>BACN,SS,APL-CDR,GM,10/14,GF,15# | BACON LAYFLAT EE 10/14 APL CDR | BACON 10/14 CT APPLE-CIDER SINGLE SLICE</t>
         </is>
       </c>
-      <c r="C336" t="inlineStr">
-        <is>
-          <t>Gluten-free sliced apple‑cider smoked bacon, 10‑14 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -5960,7 +5900,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Raw uncured sliced bacon, 13-17 slices per pound, gluten‑free</t>
+          <t>Uncured gluten-free sliced bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -6075,7 +6015,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Cooked natural bacon topping, with coating</t>
+          <t>Fully cooked natural bacon topping with coating</t>
         </is>
       </c>
     </row>
@@ -6107,11 +6047,7 @@
           <t>BACON SLICED LAYOUT 18-22 CT | BACON 18/22 CT LAYOUT HICKORY SMOKED | BACON L/O 18-22CT CC FZ</t>
         </is>
       </c>
-      <c r="C351" t="inlineStr">
-        <is>
-          <t>Frozen hickory-smoked sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -6126,7 +6062,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Fresh sliced bacon, 18-22 slices per pound, hardwood-smoked, layflat</t>
+          <t>Fresh sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -6211,7 +6147,7 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Honey-cured center cut gluten-free sliced bacon, 10-12 slices per pound, layflat</t>
+          <t>Honey-cured center-cut gluten-free sliced bacon,</t>
         </is>
       </c>
     </row>
@@ -6245,7 +6181,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Bacon end and pieces</t>
+          <t>Raw ends and pieces bacon</t>
         </is>
       </c>
     </row>
@@ -6262,7 +6198,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 13-17 slices per pound</t>
+          <t>Fully cooked sliced bacon, 13-17 or 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -6296,7 +6232,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 3/8-inch pieces</t>
+          <t>Fully cooked bacon topping, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6266,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 13-17 slices per pound</t>
+          <t>Fully cooked bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -6345,7 +6281,11 @@
           <t>BACON PRECOOKED 9/13 288 SLC | BACON PRECOOKED C/C 9/13 BCN1</t>
         </is>
       </c>
-      <c r="C365" t="inlineStr"/>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Fully cooked sliced bacon, 9-13 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">

</xml_diff>